<commit_message>
Add unit tests / Add methods to `DBReader` trait
 - Add unit tests for `excel_reader` and add excel test files
    - `Excel_DateTimeIso` stores values that is read as `calatime::Data:DateTimeIso`
    - `Excel_Merged_Cells` will be used to test for merged cells (WIP)
    - Update `Table01`
 - Add `report` module to store issues found in data_stores
 - Add methods `get_data_at`, `get_headers`, `add_issue`, and `get_issues`
 - Modify `data` field in `Cell` struct from `Result<PrimTypeData, APIError>` to `PrimTypeData`
</commit_message>
<xml_diff>
--- a/tests/assets/Table01.xlsx
+++ b/tests/assets/Table01.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">PID</t>
   </si>
@@ -31,7 +31,10 @@
     <t xml:space="preserve">Placements</t>
   </si>
   <si>
-    <t xml:space="preserve">Date</t>
+    <t xml:space="preserve">DateTime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boolean</t>
   </si>
   <si>
     <t xml:space="preserve">56b605f1-ddb7-4ff7-8180-1a5c8e11147a</t>
@@ -49,7 +52,7 @@
     <t xml:space="preserve">17e68679-2e89-4ec4-bf07-cd53ee5d7301</t>
   </si>
   <si>
-    <t xml:space="preserve">He found rain fascinating yet unpleasant. </t>
+    <t xml:space="preserve">   </t>
   </si>
   <si>
     <t xml:space="preserve">b007d97e-8938-4056-95d6-614ee49a431f</t>
@@ -98,9 +101,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
+    <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -167,7 +171,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -176,11 +180,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -307,7 +319,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34.97"/>
@@ -327,145 +339,176 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B2" s="3" t="n">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>46024</v>
+        <v>6</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>46024.05</v>
+      </c>
+      <c r="E2" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>45661</v>
+        <v>8</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>45661.2916666667</v>
+      </c>
+      <c r="E3" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>45996</v>
+        <v>10</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>45996.5416666667</v>
+      </c>
+      <c r="E4" s="5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>81</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>46000</v>
+        <v>12</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>46000.5895833333</v>
+      </c>
+      <c r="E5" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>46042</v>
+      </c>
+      <c r="E6" s="5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>97</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>45477</v>
+      </c>
+      <c r="E7" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>164</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>45102</v>
+        <v>18</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>45102.63125</v>
+      </c>
+      <c r="E8" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>67894</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D9" s="4" t="n">
         <v>45817</v>
+      </c>
+      <c r="E9" s="5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="D10" s="4" t="n">
         <v>45878</v>
+      </c>
+      <c r="E10" s="5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="D11" s="4" t="n">
         <v>45756</v>
+      </c>
+      <c r="E11" s="5" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>